<commit_message>
data: sync 12 image counts and include 56094 in degradation workbook
</commit_message>
<xml_diff>
--- a/语料库/样例数据（干净版）/无正文 降级处理/管策智研_数据清理_v1.5.xlsx
+++ b/语料库/样例数据（干净版）/无正文 降级处理/管策智研_数据清理_v1.5.xlsx
@@ -1467,7 +1467,7 @@
   <sheetPr>
     <tabColor rgb="FF92400E"/>
   </sheetPr>
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:W17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2605,6 +2605,106 @@
         <v>140</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>56094</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>edge_cases</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>白银市平川区新型城镇化建设 “十三五”发展规划</t>
+        </is>
+      </c>
+      <c r="E17" s="4">
+        <v>2939</v>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>平川区</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>区县</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>白银市</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>第十三个五年规划</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>专项规划</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>docx</t>
+        </is>
+      </c>
+      <c r="L17" s="7">
+        <v>1</v>
+      </c>
+      <c r="M17" s="7">
+        <v>0</v>
+      </c>
+      <c r="N17" s="7">
+        <v>0</v>
+      </c>
+      <c r="O17" s="7">
+        <v>0</v>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>正文为空</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>markdown缺失/07_原件或有效正文缺失/56094/56094.md</t>
+        </is>
+      </c>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>已归档第07类；干净版正文为空，原始包无可恢复DOCX原件。</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>缺少有效正文与原始文件，不能在缺少证据时生成正文。</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>正文为空</t>
+        </is>
+      </c>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>07_原件或有效正文缺失</t>
+        </is>
+      </c>
+      <c r="V17" s="5" t="inlineStr">
+        <is>
+          <t>待处理（原件或有效正文缺失）</t>
+        </is>
+      </c>
+      <c r="W17" s="5" t="inlineStr">
+        <is>
+          <t>第07类降级，待取得可靠原件后再核查。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>